<commit_message>
Fix the launch runner type error and add the skipped P0 cases.
Blob parts now use a Uint8Array so verify and the Docker build typecheck. The sheet adds the named P0 behaviours the first pass did not run, and records why the remaining ids stay under the inventory estimates.
</commit_message>
<xml_diff>
--- a/docs/test-plan/cases.xlsx
+++ b/docs/test-plan/cases.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Onboarding" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$226</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K198"/>
+  <dimension ref="A1:K226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10925,58 +10925,1542 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
+          <t>C3-12</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>Each everyday tool can be turned off on its own</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Colour, brows, beard, and nails are on</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>The owner turns one tool off and a guest requests it</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>That tool returns TOOL and the others still run after they are turned back on</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>C4-07</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>A photo over 2 MB is refused before it is decoded</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>A file larger than 2 MB</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>It is posted as the selfie</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>The API returns SIZE and does not spend a credit</t>
+        </is>
+      </c>
+      <c r="I199" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>C6-05</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Book bridal trial stores a bridal lead and a WhatsApp link</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Bridal is on and the salon has a WhatsApp number</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>The guest posts a name, a wedding date, and one look</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>A BRIDAL lead is stored and the response has a wa.me link</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>C6-06</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>A bridal trial accepts at most six looks</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Seven look ids</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>The trial is posted</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>The API returns 400</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>C9-04</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>The same bridal look is shown again without spending another try</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>A look is already in the visit cache</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>The same photo and the same selections are requested</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>The saved picture is returned and the generator is not called</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>library</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>C10-06</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>An anonymous daily cap of zero blocks the next preview</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>anonDailyCap is 0</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>A guest requests a hairstyle</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>The API returns CAP and the cap is restored to 8</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>C10-07</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>A paid preview cannot reserve a credit when the balance is zero</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>The isolation salon balance is set to 0</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>reserveCredits asks for one credit</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>It throws INSUFFICIENT and the balance stays 0</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>library</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>C11-12</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>On the way is stored on the ticket</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>A live token</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>The guest posts action way</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>onTheWay is true</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K205" s="2" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>C12-05</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>A second request for the same phone returns the open request</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>The salon is in time-request mode and one request exists</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>The same phone asks again</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>The token does not increase</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>S1-04</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>Sign out drops the staff session</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>Staff is signed in</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>They sign out</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>The queue desk redirects to login</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>S2-06</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>Start and Done move a called guest through the chair</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>One waiting guest and a free chair</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Staff taps next, start, then done</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>The public ticket goes to IN_SERVICE and then DONE</t>
+        </is>
+      </c>
+      <c r="I208" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>S3-03</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>A walk-in can be added with no phone</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>The live line is open</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>Staff adds a name and leaves the phone empty</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>The waiting card has that name and no phone</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>S3-04</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>A walk-in with a short phone is refused</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>The live line</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>The phone is 12345</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>The API returns 400</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>O1-02</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>Staff still see onboarding until the owner finishes it</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>onboardingDone is false</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>Staff open the queue desk</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>The onboarding link is present, and it is gone after Finish</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K211" s="2" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>O2-05</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>GSTIN is saved and shown back</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>The owner is signed in</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>gstin is set</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>Settings returns that value</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>O3-02</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>The owner can turn groom on and back off</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>Groom is off</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>productGroom is saved true, then false</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>The row follows both saves</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K213" s="2" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>O5-03</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>Zero is accepted as an anonymous cap and blocks that group</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>The owner saves anonDailyCap 0</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>A guest requests a preview</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>The save succeeds and the preview returns CAP</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>O9-04</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>O9</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>An inactive service disappears from the public join list</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>A service named Hidden Cut 505a</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>The owner marks it inactive</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>The public board no longer lists it</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>O11-03</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>O11</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>Almost-your-turn minutes must be from 0 to 120</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>The live desk</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>alertLeadMin is 121, then 0</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>121 is rejected and 0 is stored</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K216" s="2" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>O15-02</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>O15</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>Printing the QR on localhost is refused</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>The public URL is still this machine</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/v1/qr for the demo salon</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>The API returns LOCAL_DOMAIN</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>A2-05</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>super</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>A new salon gets a 14-day trial and a copy of the styles</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>The isolation salon was created by the super admin</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>The row and its styles are read</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>Trial end is 14 days out and every catalogue style was copied</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="K218" s="2" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>A4-04</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>super</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>A credit note is stored with the adjustment</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>The super admin adjusts by 7</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>The note is launch note 505a</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>The ledger row has that note and delta 7</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>http+db</t>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>P1-06</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>Login allows 8 attempts per email and 30 per IP in 15 minutes</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>A fresh email bucket with a limit of 8</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>The ninth attempt arrives</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>The shared limiter refuses, and the login route is wired to those two limits</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>library</t>
+        </is>
+      </c>
+      <c r="K220" s="2" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>P3-03</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>Another salon's waiting guest is not on this desk</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>The isolation salon has a waiting guest named Iso Desk Only</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>QA staff load their desk</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>That name is absent</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>http+db</t>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>P4-03</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>The guest page does not name a model or a provider</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>Mock AI</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>A guest opens the demo salon</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>The HTML has no OpenAI, gpt, or fal model name</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K222" s="2" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>X2-02</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>cross</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>No-show on the desk shows on the guest ticket</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>One waiting guest and a free chair</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>Staff call next and then no-show</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>The public ticket status is NO_SHOW</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K223" s="2" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>X7-02</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>X7</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>cross</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>The saved brand colour is on the welcome page</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>The owner sets the primary colour</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>A guest opens the welcome page</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>That colour is in the page style</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>X9-02</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>X9</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>cross</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>Resuming a salon removes the paused page</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>The isolation salon is suspended</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>Status returns to trial</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>The public page no longer says the salon is paused</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
           <t>X1-04</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
+      <c r="B226" s="2" t="inlineStr">
         <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="C198" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
         <is>
           <t>cross</t>
         </is>
       </c>
-      <c r="E198" s="2" t="inlineStr">
+      <c r="E226" s="2" t="inlineStr">
         <is>
           <t>A new live token is one higher than today's max</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F226" s="2" t="inlineStr">
         <is>
           <t>The live line has a known max token</t>
         </is>
       </c>
-      <c r="G198" s="2" t="inlineStr">
+      <c r="G226" s="2" t="inlineStr">
         <is>
           <t>Another guest joins</t>
         </is>
       </c>
-      <c r="H198" s="2" t="inlineStr">
+      <c r="H226" s="2" t="inlineStr">
         <is>
           <t>Their token is max+1</t>
         </is>
       </c>
-      <c r="I198" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J198" s="2" t="inlineStr">
-        <is>
-          <t>http</t>
-        </is>
-      </c>
-      <c r="K198" s="2" t="inlineStr"/>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>http</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K198"/>
+  <autoFilter ref="A1:K226"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>